<commit_message>
feat(data): create realistic Excel LCA workbook with multi-stage product models
</commit_message>
<xml_diff>
--- a/product_lca_template.xlsx
+++ b/product_lca_template.xlsx
@@ -19,8 +19,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+    <numFmt numFmtId="165" formatCode="0.000"/>
+  </numFmts>
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,16 +31,39 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="000F172A"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001E293B"/>
+        <bgColor rgb="001E293B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8FAFC"/>
+        <bgColor rgb="00F8FAFC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +71,53 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CBD5E1"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -416,48 +483,74 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>product_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>product_name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>functional_unit_amount</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>functional_unit</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>broom_001</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Plastic broom</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>flask_750_steel</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Insulated Stainless Steel Water Bottle (750ml)</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>unit</t>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>unit (1 reusable bottle)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>office_task_chair</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Ergonomic Office Task Chair</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>unit (1 ergonomic chair)</t>
         </is>
       </c>
     </row>
@@ -472,72 +565,188 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="23" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="49" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>process_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>product_id</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>process_name</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>stage</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>material_production</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>broom_001</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Material compounding</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>flask_raw_materials</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>flask_750_steel</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Raw Material Extraction &amp; Compounding</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Raw Materials</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>broom_manufacturing</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>broom_001</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Broom manufacturing</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>flask_manufacturing</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>flask_750_steel</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Deep-Drawing, Vacuum Brazing &amp; Flask Assembly</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>Manufacturing</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>flask_distribution</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>flask_750_steel</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Global Maritime &amp; Regional Retail Logistics</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Distribution</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>flask_end_of_life</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>flask_750_steel</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>End-of-Life Sorting &amp; Metal Scrap Recycling</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>End of Life</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>chair_materials</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>office_task_chair</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Structural Metals &amp; Polymer Injection Molding</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Raw Materials</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>chair_assembly</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>office_task_chair</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Robotic Mechanical Assembly &amp; Packaging</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Manufacturing</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>chair_logistics</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>office_task_chair</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Commercial Freight Distribution</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Distribution</t>
         </is>
       </c>
     </row>
@@ -552,158 +761,590 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="23" customWidth="1" min="1" max="1"/>
+    <col width="49" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>process_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>flow_name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>exchange_type</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>amount</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>unit</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>material_production</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Plastic granules</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>input</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>material_production</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Broom bristles</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>input</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>broom_manufacturing</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Material compounding</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>input</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>flask_raw_materials</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Steel, structural generic</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>flask_raw_materials</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Plastic granules / pellets (generic)</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>flask_raw_materials</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Copper, refined generic</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="n">
+        <v>0.008</v>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>flask_raw_materials</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Cardboard, corrugated packaging</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>flask_manufacturing</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Raw Material Extraction &amp; Compounding</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>unit</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>broom_manufacturing</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Manufacturing electricity</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>input</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="E5" t="inlineStr">
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>flask_manufacturing</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Electricity, grid average</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>kWh</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>broom_manufacturing</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>flask_manufacturing</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Process heat, from natural gas boiler</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>kWh</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>flask_manufacturing</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Tap water, municipal</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>flask_manufacturing</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>Carbon dioxide, fossil</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>output</t>
         </is>
       </c>
-      <c r="D6" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>kg</t>
+      <c r="D10" s="8" t="n">
+        <v>0.042</v>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>flask_manufacturing</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Nitrogen oxides</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>output</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>flask_distribution</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Deep-Drawing, Vacuum Brazing &amp; Flask Assembly</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>flask_end_of_life</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Global Maritime &amp; Regional Retail Logistics</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>flask_end_of_life</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Electricity, grid average</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>kWh</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>flask_end_of_life</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Carbon dioxide, fossil</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>output</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>chair_materials</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Steel, structural generic</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>chair_materials</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Aluminum, primary/secondary generic</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>chair_materials</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Plastic granules / pellets (generic)</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>chair_materials</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Cardboard, corrugated packaging</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>chair_assembly</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Structural Metals &amp; Polymer Injection Molding</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>chair_assembly</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Electricity, grid average</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>kWh</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>chair_assembly</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Carbon dioxide, fossil</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>output</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>chair_logistics</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Robotic Mechanical Assembly &amp; Packaging</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>unit</t>
         </is>
       </c>
     </row>
@@ -718,64 +1359,268 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="23" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>process_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>transport_mode</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>distance</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>distance_unit</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>transported_mass</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>mass_unit</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>broom_manufacturing</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>flask_raw_materials</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>train</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>450</v>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>km</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>flask_manufacturing</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>truck</t>
         </is>
       </c>
-      <c r="C2" t="n">
-        <v>100</v>
-      </c>
-      <c r="D2" t="inlineStr">
+      <c r="C3" s="5" t="n">
+        <v>120</v>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>km</t>
         </is>
       </c>
-      <c r="E2" t="n">
+      <c r="E3" s="9" t="n">
         <v>0.4</v>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>flask_distribution</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>ship</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>2400</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>km</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>flask_distribution</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>truck</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>180</v>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>km</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>flask_end_of_life</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>truck</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>km</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>chair_materials</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>train</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>350</v>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>km</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>chair_assembly</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>truck</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>80</v>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>km</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>chair_logistics</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>truck</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>450</v>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>km</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>kg</t>
         </is>

</xml_diff>